<commit_message>
Deduplicate shared vehicle inventory components
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-rail-freight.xlsx
+++ b/premise/data/additional_inventories/lci-rail-freight.xlsx
@@ -18974,7 +18974,7 @@
     <row r="960">
       <c r="A960" t="inlineStr">
         <is>
-          <t>carbon fiber production, weaved, at factory, carculator regional truck 2020</t>
+          <t xml:space="preserve">carbon fiber production, weaved, at factory</t>
         </is>
       </c>
       <c r="B960">
@@ -18997,12 +18997,13 @@
       </c>
       <c r="G960" t="inlineStr">
         <is>
-          <t>carbon fiber, weaved</t>
+          <t xml:space="preserve">carbon fiber, weaved</t>
         </is>
       </c>
       <c r="H960" t="inlineStr">
         <is>
-          <t>(19.873) kg / 113.169 kg dry assembly = 0.175604626709 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy. Linked to the retained canonical regional-truck component supplier.</t>
+          <t xml:space="preserve">(19.873) kg / 113.169 kg dry assembly = 0.175604626709 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy. Linked to the retained canonical regional-truck component supplier.
+Shared component reuse (2026-10-16): original model supplier 'carbon fiber production, weaved, at factory, carculator regional truck 2020' uses the existing canonical recipe in lci-carbon-fiber.xlsx; its quantities and uncertainty are retained.</t>
         </is>
       </c>
     </row>

</xml_diff>